<commit_message>
casos de chuqui corriendo
</commit_message>
<xml_diff>
--- a/data/Comparacion_BS_OBC/Mina_modelo_costo_fijo_BS/elmo_data.xlsx
+++ b/data/Comparacion_BS_OBC/Mina_modelo_costo_fijo_BS/elmo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Comparacion BS OBC\Mina_modelo_costo_fijo_BS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Comparacion_BS_OBC\Mina_modelo_costo_fijo_BS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F33BE1C4-3740-43EF-8B8F-6F008E9DFD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFCE200-E1D0-4718-9EC1-B64523432766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="136">
   <si>
     <t>id</t>
   </si>
@@ -443,6 +443,9 @@
   </si>
   <si>
     <t>Battery_swap</t>
+  </si>
+  <si>
+    <t>p_max_ssee</t>
   </si>
 </sst>
 </file>
@@ -2756,14 +2759,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D86F6B0-26ED-4B02-B890-EDAFE42B3137}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2785,8 +2788,11 @@
       <c r="G1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2808,8 +2814,11 @@
       <c r="G2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2831,8 +2840,11 @@
       <c r="G3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2854,8 +2866,11 @@
       <c r="G4">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2876,6 +2891,9 @@
       </c>
       <c r="G5">
         <v>4</v>
+      </c>
+      <c r="H5">
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>